<commit_message>
funciona mantenimiento flata esa gregar el paso de verificacion a la c223
</commit_message>
<xml_diff>
--- a/temp_mhr/asignar_plan_53069917.xlsx
+++ b/temp_mhr/asignar_plan_53069917.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,330 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>700179566</t>
+          <t>700157006</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>501136801</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>700045114</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>501045644</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>700176964</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>501155859</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>700156860</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>501136715</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>700171838</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>501150933</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>700171837</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>501150932</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>700176669</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>501155554</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>700167072</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>501146077</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>700167975</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>501147010</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>700178545</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>501157420</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
por si la cago antes de tirarmelo
</commit_message>
<xml_diff>
--- a/temp_mhr/asignar_plan_53069917.xlsx
+++ b/temp_mhr/asignar_plan_53069917.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>700157006</t>
+          <t>700179478</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>501136801</t>
+          <t>501158343</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>700045114</t>
+          <t>700077429</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>501045644</t>
+          <t>501036082</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>700176964</t>
+          <t>700177912</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>501155859</t>
+          <t>501156817</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>700156860</t>
+          <t>700175831</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>501136715</t>
+          <t>501155006</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>700171838</t>
+          <t>700178576</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>501150933</t>
+          <t>501157441</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>700171837</t>
+          <t>700161977</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>501150932</t>
+          <t>501141943</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>700176669</t>
+          <t>700176938</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>501155554</t>
+          <t>501155833</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>700167072</t>
+          <t>700178544</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>501146077</t>
+          <t>501157419</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>700167975</t>
+          <t>700171837</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>501147010</t>
+          <t>501150932</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>700178545</t>
+          <t>700157007</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,2897 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
+          <t>501136802</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>700178410</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>501157275</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>700178203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>501157068</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>700157233</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>501137329</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>700156861</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>501136716</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>700158999</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>501138843</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>700180394</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>501159281</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>700178386</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>501157251</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>700157235</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>501137331</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>700178411</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>501157276</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>700071403</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>501033761</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>700161780</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>501141455</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>700161976</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>501141942</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>700071580</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>501033978</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>700179566</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>501158431</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>700178423</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>501157288</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>700167083</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>501146098</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>700157237</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>501137333</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>700177340</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>501156245</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>700161978</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>501141944</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>700175860</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>501155035</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>700176671</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>501155556</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>700175832</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>501155007</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>700027910</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>501031035</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>700163027</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>501142962</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>701126709</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>501104964</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>700175772</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>501155781</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>700176964</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>501155859</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>700027936</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>501031061</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>700071404</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>501033762</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>700178545</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
           <t>501157420</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>700178424</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>501157289</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>700071534</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>501033912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>700175771</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>501155780</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>700157238</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>501137334</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>700179567</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>501158432</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>700171838</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>501150933</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>700179435</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>501158300</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>700156860</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>501136715</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>700177313</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>501156218</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>700045114</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>501045644</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>700175861</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>501155036</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>700077428</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>501036081</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>700071533</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>501033911</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>700154329</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>501134404</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>700161779</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>501141454</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>700176670</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>501155555</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>700172749</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>501151855</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>700167975</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>501147010</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>700040953</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>501040053</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>700177060</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>501155955</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>700177059</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>501155954</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>700177911</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>501156816</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>700174255</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>501153390</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>700175770</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>501155779</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>700133588</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>501114011</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>700163028</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>501142963</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>700133587</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>501114010</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>700174254</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>501153389</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>700176963</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>501155858</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>700165944</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>501144949</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>700180597</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>501159492</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>700178192</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>501157057</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>700157234</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>501137330</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>700175780</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>501154955</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>700176668</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>501155553</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>700027935</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>501031060</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>700167138</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>501146143</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>700027911</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>501031036</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>700153345</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>501133530</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>700040952</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>501040052</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>700175773</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>501155783</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>700168256</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>501147301</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>700167072</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>501146077</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>700179436</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>501158301</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>700177732</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>501156637</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>700179544</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>501158419</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>700177314</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>501156219</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>700176937</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>501155832</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>700157236</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>501137332</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>700154328</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>501134403</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>700157006</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>501136801</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>700161979</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>501141945</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>700176669</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>501155554</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>700179219</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>501158084</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>701126710</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>53064821</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>501104965</t>
         </is>
       </c>
     </row>

</xml_diff>